<commit_message>
test(QLPT-347): record EP execution results
</commit_message>
<xml_diff>
--- a/postman/EP/Nhan/QLPT-347/QLPT-347-EP-Test-Cases.xlsx
+++ b/postman/EP/Nhan/QLPT-347/QLPT-347-EP-Test-Cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc65ff1765efc41c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cart EP" sheetId="2" r:id="R999a7aaddbd84b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion EP" sheetId="3" r:id="R58ae3be4e82c4184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rda225ed9727a455b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cart EP" sheetId="2" r:id="Rff0aae92aab2418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion EP" sheetId="3" r:id="R480733f90cc24b8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,7 +578,7 @@
       </x:c>
       <x:c r="E5" s="48" t="n">
         <x:f>COUNTIF('Cart EP'!T2:T200,"PASS")+COUNTIF('Promotion EP'!T2:T200,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F5" s="47"/>
       <x:c r="G5" s="47"/>
@@ -616,7 +616,7 @@
       </x:c>
       <x:c r="E7" s="50" t="n">
         <x:f>COUNTIF('Cart EP'!T2:T200,"NOT RUN")+COUNTIF('Promotion EP'!T2:T200,"NOT RUN")</x:f>
-        <x:v>37</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="47"/>
       <x:c r="G7" s="47"/>
@@ -628,7 +628,7 @@
       </x:c>
       <x:c r="B8" s="31" t="str">
         <x:f>IF(E6&gt;0,"FAIL",IF(E7&gt;0,"NOT RUN","PASS"))</x:f>
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C8" s="39"/>
       <x:c r="D8" s="39"/>
@@ -692,7 +692,7 @@
       </x:c>
       <x:c r="F11" s="51" t="n">
         <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G11" s="51" t="n">
         <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"FAIL")</x:f>
@@ -700,7 +700,7 @@
       </x:c>
       <x:c r="H11" s="51" t="n">
         <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"NOT RUN")</x:f>
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -722,7 +722,7 @@
       </x:c>
       <x:c r="F12" s="52" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G12" s="52" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"FAIL")</x:f>
@@ -730,7 +730,7 @@
       </x:c>
       <x:c r="H12" s="52" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"NOT RUN")</x:f>
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -752,7 +752,7 @@
       </x:c>
       <x:c r="F13" s="51" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"PASS")</x:f>
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G13" s="51" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"FAIL")</x:f>
@@ -760,7 +760,7 @@
       </x:c>
       <x:c r="H13" s="51" t="n">
         <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"NOT RUN")</x:f>
-        <x:v>14</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -942,10 +942,14 @@
       <x:c r="Q2" s="11" t="str">
         <x:v>HTTP 200; tạo đúng một cart item quantity=5, subtotal đúng và không trừ tồn kho.</x:v>
       </x:c>
-      <x:c r="R2" s="11"/>
-      <x:c r="S2" s="11"/>
+      <x:c r="R2" s="11" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S2" s="11" t="str">
+        <x:v>HTTP 200; 7/7 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T2" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U2" s="11"/>
     </x:row>
@@ -1002,10 +1006,14 @@
       <x:c r="Q3" s="12" t="str">
         <x:v>HTTP 400; không tạo item và trạng thái giỏ không đổi.</x:v>
       </x:c>
-      <x:c r="R3" s="12"/>
-      <x:c r="S3" s="12"/>
+      <x:c r="R3" s="12" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S3" s="12" t="str">
+        <x:v>HTTP 400; 5/5 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T3" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U3" s="12"/>
     </x:row>
@@ -1062,10 +1070,14 @@
       <x:c r="Q4" s="11" t="str">
         <x:v>HTTP 400; không tạo item khi quantity vượt stockQty=10.</x:v>
       </x:c>
-      <x:c r="R4" s="11"/>
-      <x:c r="S4" s="11"/>
+      <x:c r="R4" s="11" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S4" s="11" t="str">
+        <x:v>HTTP 400; 5/5 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T4" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U4" s="11"/>
     </x:row>
@@ -1122,10 +1134,14 @@
       <x:c r="Q5" s="12" t="str">
         <x:v>HTTP 400 do @NotNull; giỏ không thay đổi.</x:v>
       </x:c>
-      <x:c r="R5" s="12"/>
-      <x:c r="S5" s="12"/>
+      <x:c r="R5" s="12" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S5" s="12" t="str">
+        <x:v>HTTP 400; 5/5 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T5" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U5" s="12"/>
     </x:row>
@@ -1182,10 +1198,14 @@
       <x:c r="Q6" s="11" t="str">
         <x:v>HTTP 400 do quantity không ánh xạ hợp lệ vào Integer; giỏ không thay đổi.</x:v>
       </x:c>
-      <x:c r="R6" s="11"/>
-      <x:c r="S6" s="11"/>
+      <x:c r="R6" s="11" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S6" s="11" t="str">
+        <x:v>HTTP 400; 5/5 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T6" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U6" s="11"/>
     </x:row>
@@ -1242,10 +1262,14 @@
       <x:c r="Q7" s="12" t="str">
         <x:v>HTTP 200; cart item được cập nhật quantity=5, subtotal đúng, kho không đổi.</x:v>
       </x:c>
-      <x:c r="R7" s="12"/>
-      <x:c r="S7" s="12"/>
+      <x:c r="R7" s="12" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S7" s="12" t="str">
+        <x:v>HTTP 200; 7/7 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T7" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U7" s="12"/>
     </x:row>
@@ -1302,10 +1326,14 @@
       <x:c r="Q8" s="11" t="str">
         <x:v>HTTP 400; cart item giữ quantity baseline.</x:v>
       </x:c>
-      <x:c r="R8" s="11"/>
-      <x:c r="S8" s="11"/>
+      <x:c r="R8" s="11" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S8" s="11" t="str">
+        <x:v>HTTP 400; 6/6 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T8" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U8" s="11"/>
     </x:row>
@@ -1362,10 +1390,14 @@
       <x:c r="Q9" s="12" t="str">
         <x:v>HTTP 400; cart item giữ quantity baseline.</x:v>
       </x:c>
-      <x:c r="R9" s="12"/>
-      <x:c r="S9" s="12"/>
+      <x:c r="R9" s="12" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S9" s="12" t="str">
+        <x:v>HTTP 400; 6/6 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T9" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U9" s="12"/>
     </x:row>
@@ -1422,10 +1454,14 @@
       <x:c r="Q10" s="11" t="str">
         <x:v>HTTP 200; vẫn một item, quantity sau cộng dồn bằng 9 và kho không đổi.</x:v>
       </x:c>
-      <x:c r="R10" s="11"/>
-      <x:c r="S10" s="11"/>
+      <x:c r="R10" s="11" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S10" s="11" t="str">
+        <x:v>HTTP 200; 7/7 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T10" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U10" s="11"/>
     </x:row>
@@ -1482,10 +1518,14 @@
       <x:c r="Q11" s="12" t="str">
         <x:v>HTTP 400; quantity vẫn bằng baseline 8.</x:v>
       </x:c>
-      <x:c r="R11" s="12"/>
-      <x:c r="S11" s="12"/>
+      <x:c r="R11" s="12" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S11" s="12" t="str">
+        <x:v>HTTP 400; 6/6 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T11" s="13" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U11" s="12"/>
     </x:row>
@@ -1647,10 +1687,14 @@
       <x:c r="Q2" s="53" t="str">
         <x:v>Admin tạo HTTP 201; Customer apply HTTP 200; discount=floor(subtotal×50/100).</x:v>
       </x:c>
-      <x:c r="R2" s="53"/>
-      <x:c r="S2" s="53"/>
+      <x:c r="R2" s="53" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S2" s="53" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T2" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U2" s="53"/>
     </x:row>
@@ -1707,10 +1751,14 @@
       <x:c r="Q3" s="54" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R3" s="54"/>
-      <x:c r="S3" s="54"/>
+      <x:c r="R3" s="54" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S3" s="54" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T3" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U3" s="54"/>
     </x:row>
@@ -1767,10 +1815,14 @@
       <x:c r="Q4" s="53" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R4" s="53"/>
-      <x:c r="S4" s="53"/>
+      <x:c r="R4" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S4" s="53" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T4" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U4" s="53"/>
     </x:row>
@@ -1827,10 +1879,14 @@
       <x:c r="Q5" s="54" t="str">
         <x:v>Admin trả HTTP 400 do value bắt buộc.</x:v>
       </x:c>
-      <x:c r="R5" s="54"/>
-      <x:c r="S5" s="54"/>
+      <x:c r="R5" s="54" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S5" s="54" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T5" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U5" s="54"/>
     </x:row>
@@ -1887,10 +1943,14 @@
       <x:c r="Q6" s="53" t="str">
         <x:v>Admin tạo HTTP 201; apply HTTP 200; discount=value và tổng còn 0.01.</x:v>
       </x:c>
-      <x:c r="R6" s="53"/>
-      <x:c r="S6" s="53"/>
+      <x:c r="R6" s="53" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S6" s="53" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T6" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U6" s="53"/>
     </x:row>
@@ -1947,10 +2007,14 @@
       <x:c r="Q7" s="54" t="str">
         <x:v>Admin tạo HTTP 201; apply HTTP 200; discount=subtotal và totalAfterDiscount=0.</x:v>
       </x:c>
-      <x:c r="R7" s="54"/>
-      <x:c r="S7" s="54"/>
+      <x:c r="R7" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S7" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T7" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U7" s="54"/>
     </x:row>
@@ -2007,10 +2071,14 @@
       <x:c r="Q8" s="53" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R8" s="53"/>
-      <x:c r="S8" s="53"/>
+      <x:c r="R8" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S8" s="53" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T8" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U8" s="53"/>
     </x:row>
@@ -2067,10 +2135,14 @@
       <x:c r="Q9" s="54" t="str">
         <x:v>Admin tạo HTTP 201; Customer có thể áp dụng khi các điều kiện khác hợp lệ.</x:v>
       </x:c>
-      <x:c r="R9" s="54"/>
-      <x:c r="S9" s="54"/>
+      <x:c r="R9" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S9" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T9" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U9" s="54"/>
     </x:row>
@@ -2127,10 +2199,14 @@
       <x:c r="Q10" s="53" t="str">
         <x:v>Admin tạo HTTP 201 và lưu đúng minOrderValue.</x:v>
       </x:c>
-      <x:c r="R10" s="53"/>
-      <x:c r="S10" s="53"/>
+      <x:c r="R10" s="53" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S10" s="53" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T10" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U10" s="53"/>
     </x:row>
@@ -2187,10 +2263,14 @@
       <x:c r="Q11" s="54" t="str">
         <x:v>Admin tạo HTTP 201; response lưu minOrderValue=0; Customer apply HTTP 200 khi các điều kiện khác hợp lệ.</x:v>
       </x:c>
-      <x:c r="R11" s="54"/>
-      <x:c r="S11" s="54"/>
+      <x:c r="R11" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S11" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T11" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U11" s="54"/>
     </x:row>
@@ -2247,10 +2327,14 @@
       <x:c r="Q12" s="53" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R12" s="53"/>
-      <x:c r="S12" s="53"/>
+      <x:c r="R12" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S12" s="53" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T12" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U12" s="53"/>
     </x:row>
@@ -2307,10 +2391,14 @@
       <x:c r="Q13" s="54" t="str">
         <x:v>Apply trả HTTP 400; không tăng lượt sử dụng.</x:v>
       </x:c>
-      <x:c r="R13" s="54"/>
-      <x:c r="S13" s="54"/>
+      <x:c r="R13" s="54" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S13" s="54" t="str">
+        <x:v>HTTP 400; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T13" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U13" s="54"/>
     </x:row>
@@ -2367,10 +2455,14 @@
       <x:c r="Q14" s="55" t="str">
         <x:v>Apply trả HTTP 200; discount và total tính đúng; preview không tăng lượt.</x:v>
       </x:c>
-      <x:c r="R14" s="55"/>
-      <x:c r="S14" s="55"/>
+      <x:c r="R14" s="55" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S14" s="55" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T14" s="58" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U14" s="55"/>
     </x:row>
@@ -2427,10 +2519,14 @@
       <x:c r="Q15" s="54" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R15" s="54"/>
-      <x:c r="S15" s="54"/>
+      <x:c r="R15" s="54" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S15" s="54" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T15" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U15" s="54"/>
     </x:row>
@@ -2487,10 +2583,14 @@
       <x:c r="Q16" s="53" t="str">
         <x:v>Admin tạo HTTP 201; lưu maxUses=1; mã mới còn lượt.</x:v>
       </x:c>
-      <x:c r="R16" s="53"/>
-      <x:c r="S16" s="53"/>
+      <x:c r="R16" s="53" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S16" s="53" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T16" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U16" s="53"/>
     </x:row>
@@ -2547,10 +2647,14 @@
       <x:c r="Q17" s="54" t="str">
         <x:v>Admin tạo HTTP 201; maxUses=null và mã dùng được.</x:v>
       </x:c>
-      <x:c r="R17" s="54"/>
-      <x:c r="S17" s="54"/>
+      <x:c r="R17" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S17" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T17" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U17" s="54"/>
     </x:row>
@@ -2607,10 +2711,14 @@
       <x:c r="Q18" s="53" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R18" s="53"/>
-      <x:c r="S18" s="53"/>
+      <x:c r="R18" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S18" s="53" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T18" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U18" s="53"/>
     </x:row>
@@ -2667,10 +2775,14 @@
       <x:c r="Q19" s="54" t="str">
         <x:v>Admin tạo HTTP 201; lưu maxUsesPerUser=1; user chưa dùng nên mã hợp lệ.</x:v>
       </x:c>
-      <x:c r="R19" s="54"/>
-      <x:c r="S19" s="54"/>
+      <x:c r="R19" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S19" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T19" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U19" s="54"/>
     </x:row>
@@ -2727,10 +2839,14 @@
       <x:c r="Q20" s="53" t="str">
         <x:v>Admin tạo HTTP 201; maxUsesPerUser=null và mã dùng được.</x:v>
       </x:c>
-      <x:c r="R20" s="53"/>
-      <x:c r="S20" s="53"/>
+      <x:c r="R20" s="53" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S20" s="53" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T20" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U20" s="53"/>
     </x:row>
@@ -2787,10 +2903,14 @@
       <x:c r="Q21" s="54" t="str">
         <x:v>Admin tạo HTTP 201 và lưu đúng hai giới hạn.</x:v>
       </x:c>
-      <x:c r="R21" s="54"/>
-      <x:c r="S21" s="54"/>
+      <x:c r="R21" s="54" t="n">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="S21" s="54" t="str">
+        <x:v>HTTP 201; 11/11 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T21" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U21" s="54"/>
     </x:row>
@@ -2847,10 +2967,14 @@
       <x:c r="Q22" s="53" t="str">
         <x:v>Admin trả HTTP 400 và không tạo promotion.</x:v>
       </x:c>
-      <x:c r="R22" s="53"/>
-      <x:c r="S22" s="53"/>
+      <x:c r="R22" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S22" s="53" t="str">
+        <x:v>HTTP 400; 2/2 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T22" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U22" s="53"/>
     </x:row>
@@ -2907,10 +3031,14 @@
       <x:c r="Q23" s="54" t="str">
         <x:v>Apply trả HTTP 200; preview không tăng usedCount.</x:v>
       </x:c>
-      <x:c r="R23" s="54"/>
-      <x:c r="S23" s="54"/>
+      <x:c r="R23" s="54" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S23" s="54" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T23" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U23" s="54"/>
     </x:row>
@@ -2967,10 +3095,14 @@
       <x:c r="Q24" s="53" t="str">
         <x:v>Apply trả HTTP 400; preview không tăng usedCount.</x:v>
       </x:c>
-      <x:c r="R24" s="53"/>
-      <x:c r="S24" s="53"/>
+      <x:c r="R24" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S24" s="53" t="str">
+        <x:v>HTTP 400; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T24" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U24" s="53"/>
     </x:row>
@@ -3027,10 +3159,14 @@
       <x:c r="Q25" s="54" t="str">
         <x:v>Apply trả HTTP 200; preview không tạo thêm usage.</x:v>
       </x:c>
-      <x:c r="R25" s="54"/>
-      <x:c r="S25" s="54"/>
+      <x:c r="R25" s="54" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S25" s="54" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T25" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U25" s="54"/>
     </x:row>
@@ -3087,10 +3223,14 @@
       <x:c r="Q26" s="53" t="str">
         <x:v>Apply trả HTTP 400; không tạo thêm usage.</x:v>
       </x:c>
-      <x:c r="R26" s="53"/>
-      <x:c r="S26" s="53"/>
+      <x:c r="R26" s="53" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S26" s="53" t="str">
+        <x:v>HTTP 400; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T26" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U26" s="53"/>
     </x:row>
@@ -3147,10 +3287,14 @@
       <x:c r="Q27" s="54" t="str">
         <x:v>Available trả HTTP 200 và không chứa promotion fixture.</x:v>
       </x:c>
-      <x:c r="R27" s="54"/>
-      <x:c r="S27" s="54"/>
+      <x:c r="R27" s="54" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S27" s="54" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T27" s="57" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U27" s="54"/>
     </x:row>
@@ -3207,10 +3351,14 @@
       <x:c r="Q28" s="56" t="str">
         <x:v>Available trả HTTP 200; promotion có isEligible=false và reason không rỗng.</x:v>
       </x:c>
-      <x:c r="R28" s="56"/>
-      <x:c r="S28" s="56"/>
+      <x:c r="R28" s="56" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S28" s="56" t="str">
+        <x:v>HTTP 200; 4/4 kiểm tra PASS; hành vi và trạng thái dữ liệu khớp Expected Result.</x:v>
+      </x:c>
       <x:c r="T28" s="59" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="U28" s="56"/>
     </x:row>

</xml_diff>

<commit_message>
test(QLPT-347): add Product EP coverage
</commit_message>
<xml_diff>
--- a/postman/EP/Nhan/QLPT-347/QLPT-347-EP-Test-Cases.xlsx
+++ b/postman/EP/Nhan/QLPT-347/QLPT-347-EP-Test-Cases.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rda225ed9727a455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cart EP" sheetId="2" r:id="Rff0aae92aab2418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion EP" sheetId="3" r:id="R480733f90cc24b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3ffe1b7c2c91465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cart EP" sheetId="2" r:id="R13f65a466e2f47bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Promotion EP" sheetId="3" r:id="Rc0715b87df9e4bbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product EP" sheetId="4" r:id="R673ecde0884346e2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -558,8 +559,7 @@
         <x:v>Tổng testcase</x:v>
       </x:c>
       <x:c r="E4" s="46" t="n">
-        <x:f>COUNTA('Cart EP'!B2:B200)+COUNTA('Promotion EP'!B2:B200)</x:f>
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="F4" s="47"/>
       <x:c r="G4" s="47"/>
@@ -570,15 +570,14 @@
         <x:v>Phạm vi</x:v>
       </x:c>
       <x:c r="B5" s="31" t="str">
-        <x:v>Cart quantity; Promotion value/minimum order; Promotion usage limits</x:v>
+        <x:v>Product stock/price filters; Cart quantity; Promotion value/minimum order; Promotion usage limits</x:v>
       </x:c>
       <x:c r="C5" s="39"/>
       <x:c r="D5" s="41" t="str">
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="E5" s="48" t="n">
-        <x:f>COUNTIF('Cart EP'!T2:T200,"PASS")+COUNTIF('Promotion EP'!T2:T200,"PASS")</x:f>
-        <x:v>37</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="F5" s="47"/>
       <x:c r="G5" s="47"/>
@@ -596,7 +595,6 @@
         <x:v>FAIL</x:v>
       </x:c>
       <x:c r="E6" s="49" t="n">
-        <x:f>COUNTIF('Cart EP'!T2:T200,"FAIL")+COUNTIF('Promotion EP'!T2:T200,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="47"/>
@@ -615,7 +613,6 @@
         <x:v>NOT RUN</x:v>
       </x:c>
       <x:c r="E7" s="50" t="n">
-        <x:f>COUNTIF('Cart EP'!T2:T200,"NOT RUN")+COUNTIF('Promotion EP'!T2:T200,"NOT RUN")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="47"/>
@@ -675,103 +672,107 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32" t="str">
-        <x:v>QLPT-350</x:v>
+        <x:v>QLPT-347</x:v>
       </x:c>
       <x:c r="B11" s="32" t="str">
-        <x:v>Cart quantity</x:v>
+        <x:v>Product stock/price filters</x:v>
       </x:c>
       <x:c r="C11" s="32" t="str">
-        <x:v>Integer 1..S; tổng quantity &lt;= S</x:v>
+        <x:v>stockQty = 0 hoặc &gt;0; minPrice/maxPrice bao gồm hoặc loại fixture; tham số giá bỏ trống</x:v>
       </x:c>
       <x:c r="D11" s="32" t="str">
-        <x:v>&lt;1; &gt;S; null; decimal; tổng &gt;S</x:v>
+        <x:v>minPrice/maxPrice sai kiểu dữ liệu</x:v>
       </x:c>
       <x:c r="E11" s="51" t="n">
-        <x:f>COUNTIF('Cart EP'!D2:D200,A11)</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F11" s="51" t="n">
-        <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"PASS")</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" s="51" t="n">
-        <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" s="51" t="n">
-        <x:f>COUNTIFS('Cart EP'!D2:D200,A11,'Cart EP'!T2:T200,"NOT RUN")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="31" t="str">
-        <x:v>QLPT-351</x:v>
+        <x:v>QLPT-350</x:v>
       </x:c>
       <x:c r="B12" s="31" t="str">
-        <x:v>Promotion value/minimum</x:v>
+        <x:v>Cart quantity</x:v>
       </x:c>
       <x:c r="C12" s="31" t="str">
-        <x:v>PERCENT 0.01..100; FIXED &gt;=0.01; minOrder &gt;=0</x:v>
+        <x:v>Integer 1..S; tổng quantity &lt;= S</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
-        <x:v>null; value ngoài miền; minOrder &lt;0; subtotal &lt; minimum</x:v>
+        <x:v>&lt;1; &gt;S; null; decimal; tổng &gt;S</x:v>
       </x:c>
       <x:c r="E12" s="52" t="n">
-        <x:f>COUNTIF('Promotion EP'!D2:D200,A12)</x:f>
-        <x:v>13</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F12" s="52" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"PASS")</x:f>
-        <x:v>13</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G12" s="52" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"FAIL")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="52" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A12,'Promotion EP'!T2:T200,"NOT RUN")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32" t="str">
+        <x:v>QLPT-351</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>Promotion value/minimum</x:v>
+      </x:c>
+      <x:c r="C13" s="32" t="str">
+        <x:v>PERCENT 0.01..100; FIXED &gt;=0.01; minOrder &gt;=0</x:v>
+      </x:c>
+      <x:c r="D13" s="32" t="str">
+        <x:v>null; value ngoài miền; minOrder &lt;0; subtotal &lt; minimum</x:v>
+      </x:c>
+      <x:c r="E13" s="51" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="F13" s="51" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G13" s="51" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="51" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="39" t="str">
         <x:v>QLPT-352</x:v>
       </x:c>
-      <x:c r="B13" s="32" t="str">
+      <x:c r="B14" s="39" t="str">
         <x:v>Promotion usage limits</x:v>
       </x:c>
-      <x:c r="C13" s="32" t="str">
+      <x:c r="C14" s="39" t="str">
         <x:v>null hoặc &gt;=1; còn lượt; per-user &lt;= total</x:v>
       </x:c>
-      <x:c r="D13" s="32" t="str">
+      <x:c r="D14" s="39" t="str">
         <x:v>&lt;=0; hết lượt; per-user &gt; total</x:v>
       </x:c>
-      <x:c r="E13" s="51" t="n">
-        <x:f>COUNTIF('Promotion EP'!D2:D200,A13)</x:f>
+      <x:c r="E14" s="39" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="F13" s="51" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"PASS")</x:f>
+      <x:c r="F14" s="39" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="G13" s="51" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"FAIL")</x:f>
+      <x:c r="G14" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H13" s="51" t="n">
-        <x:f>COUNTIFS('Promotion EP'!D2:D200,A13,'Promotion EP'!T2:T200,"NOT RUN")</x:f>
+      <x:c r="H14" s="39" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="39"/>
-      <x:c r="B14" s="39"/>
-      <x:c r="C14" s="39"/>
-      <x:c r="D14" s="39"/>
-      <x:c r="E14" s="39"/>
-      <x:c r="F14" s="39"/>
-      <x:c r="G14" s="39"/>
-      <x:c r="H14" s="39"/>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="37" t="str">
@@ -3370,4 +3371,677 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>No.</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>TC ID</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Module</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Requirement ID</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Function</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>Test Basis</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>Test Technique</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>Input Field</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>Equivalence Classes</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>Selected Partition</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>Preconditions / Steps</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>Test Data</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>Representative Value</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>Expected HTTP Status</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="R1" t="str">
+        <x:v>Actual HTTP Status</x:v>
+      </x:c>
+      <x:c r="S1" t="str">
+        <x:v>Actual Result</x:v>
+      </x:c>
+      <x:c r="T1" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="U1" t="str">
+        <x:v>Bug ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>PROD-EP-STOCK-ZERO</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Đọc sản phẩm thuộc lớp hết hàng</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>/api/products/{slug}</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>stockQty (dữ liệu fixture)</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>Hết hàng: stockQty = 0; Còn hàng: stockQty &gt; 0</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>Hết hàng: stockQty = 0</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>{{zero_product_slug}}</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P2" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>HTTP 200; trả đúng variant có stockQty=0 và không thay đổi tồn kho.</x:v>
+      </x:c>
+      <x:c r="R2" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S2" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; đúng product và stockQty=0.</x:v>
+      </x:c>
+      <x:c r="T2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>PROD-EP-STOCK-POSITIVE</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Đọc sản phẩm thuộc lớp còn hàng</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>/api/products/{slug}</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>stockQty (dữ liệu fixture)</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>Hết hàng: stockQty = 0; Còn hàng: stockQty &gt; 0</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>Còn hàng: stockQty &gt; 0</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>{{product_slug}}</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="P3" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>HTTP 200; trả đúng variant có stockQty&gt;0 và không thay đổi tồn kho.</x:v>
+      </x:c>
+      <x:c r="R3" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S3" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; đúng product và stockQty=10.</x:v>
+      </x:c>
+      <x:c r="T3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>PROD-EP-MIN-INCLUDE</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Lọc minPrice thuộc lớp bao gồm sản phẩm</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>/api/products?keyword={name}&amp;minPrice={value}</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>minPrice</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Bao gồm fixture: minPrice &lt;= S; Loại fixture: minPrice &gt; S; Không hợp lệ: sai kiểu</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Hợp lệ: minPrice &lt; S</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>minPrice = S - 1</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>S - 1 = 18,999</x:v>
+      </x:c>
+      <x:c r="P4" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>HTTP 200; danh sách chứa product fixture có giá S.</x:v>
+      </x:c>
+      <x:c r="R4" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S4" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; nhận 1 sản phẩm và có product fixture.</x:v>
+      </x:c>
+      <x:c r="T4" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>PROD-EP-MIN-EXCLUDE</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Lọc minPrice thuộc lớp loại sản phẩm</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>/api/products?keyword={name}&amp;minPrice={value}</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>minPrice</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>Bao gồm fixture: minPrice &lt;= S; Loại fixture: minPrice &gt; S; Không hợp lệ: sai kiểu</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>Hợp lệ: minPrice &gt; S</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>minPrice = S + 1</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>S + 1 = 19,001</x:v>
+      </x:c>
+      <x:c r="P5" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>HTTP 200; danh sách không chứa product fixture có giá S.</x:v>
+      </x:c>
+      <x:c r="R5" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S5" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; nhận 0 sản phẩm, fixture bị loại đúng.</x:v>
+      </x:c>
+      <x:c r="T5" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>PROD-EP-MAX-EXCLUDE</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Lọc maxPrice thuộc lớp loại sản phẩm</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>/api/products?keyword={name}&amp;maxPrice={value}</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>maxPrice</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Bao gồm fixture: maxPrice &gt;= S; Loại fixture: maxPrice &lt; S; Không hợp lệ: sai kiểu</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Hợp lệ: maxPrice &lt; S</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>maxPrice = S - 1</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>S - 1 = 18,999</x:v>
+      </x:c>
+      <x:c r="P6" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>HTTP 200; danh sách không chứa product fixture có giá S.</x:v>
+      </x:c>
+      <x:c r="R6" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S6" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; nhận 0 sản phẩm, fixture bị loại đúng.</x:v>
+      </x:c>
+      <x:c r="T6" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>PROD-EP-MAX-INCLUDE</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Lọc maxPrice thuộc lớp bao gồm sản phẩm</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>/api/products?keyword={name}&amp;maxPrice={value}</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>maxPrice</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>Bao gồm fixture: maxPrice &gt;= S; Loại fixture: maxPrice &lt; S; Không hợp lệ: sai kiểu</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>Hợp lệ: maxPrice &gt; S</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>maxPrice = S + 1</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>S + 1 = 19,001</x:v>
+      </x:c>
+      <x:c r="P7" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>HTTP 200; danh sách chứa product fixture có giá S.</x:v>
+      </x:c>
+      <x:c r="R7" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S7" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; nhận 1 sản phẩm và có product fixture.</x:v>
+      </x:c>
+      <x:c r="T7" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>PROD-EP-PRICE-OMITTED</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Lọc sản phẩm khi bỏ tham số giá</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>/api/products?keyword={name}</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>minPrice/maxPrice</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>Có tham số giá hợp lệ; Không truyền tham số giá; Tham số sai kiểu</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>Hợp lệ: không truyền minPrice/maxPrice</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>Không gửi minPrice và maxPrice</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>omitted</x:v>
+      </x:c>
+      <x:c r="P8" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="Q8" t="str">
+        <x:v>HTTP 200; không áp dụng điều kiện giá và vẫn trả product fixture.</x:v>
+      </x:c>
+      <x:c r="R8" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="S8" t="str">
+        <x:v>HTTP 200; 3/3 kiểm tra PASS; nhận 1 sản phẩm và có product fixture.</x:v>
+      </x:c>
+      <x:c r="T8" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>PROD-EP-MIN-MALFORMED</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Từ chối minPrice sai kiểu dữ liệu</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>/api/products?minPrice={value}</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>minPrice</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>Hợp lệ: số chuyển được sang BigDecimal; Không hợp lệ: chuỗi không phải số</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>Không hợp lệ: minPrice sai kiểu</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>minPrice=abc</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>abc</x:v>
+      </x:c>
+      <x:c r="P9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>HTTP 400 do không chuyển đổi được minPrice sang BigDecimal.</x:v>
+      </x:c>
+      <x:c r="R9" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S9" t="str">
+        <x:v>HTTP 400; 1/1 kiểm tra PASS; API từ chối giá trị không chuyển đổi được sang BigDecimal.</x:v>
+      </x:c>
+      <x:c r="T9" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>PROD-EP-MAX-MALFORMED</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Product</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>QLPT-347</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Từ chối maxPrice sai kiểu dữ liệu</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>/api/products?maxPrice={value}</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>ProductFilterRequest định nghĩa minPrice/maxPrice kiểu BigDecimal; ProductServiceImpl.buildSpec áp dụng salePrice &gt;= minPrice và salePrice &lt;= maxPrice; ProductMapper trả stockQty của variant.
+https://hientm0978.atlassian.net/browse/QLPT-347</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Equivalence Partitioning</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>maxPrice</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Hợp lệ: số chuyển được sang BigDecimal; Không hợp lệ: chuỗi không phải số</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>Không hợp lệ: maxPrice sai kiểu</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>Fixture Product active, slug/id và giá khớp environment local. Các ca chỉ gửi GET và không làm thay đổi dữ liệu.</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>maxPrice=abc</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>abc</x:v>
+      </x:c>
+      <x:c r="P10" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>HTTP 400 do không chuyển đổi được maxPrice sang BigDecimal.</x:v>
+      </x:c>
+      <x:c r="R10" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="S10" t="str">
+        <x:v>HTTP 400; 1/1 kiểm tra PASS; API từ chối giá trị không chuyển đổi được sang BigDecimal.</x:v>
+      </x:c>
+      <x:c r="T10" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="U10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11"/>
+      <x:c r="L11"/>
+      <x:c r="M11"/>
+      <x:c r="N11"/>
+      <x:c r="O11"/>
+      <x:c r="P11"/>
+      <x:c r="Q11"/>
+      <x:c r="R11"/>
+      <x:c r="S11"/>
+      <x:c r="T11"/>
+      <x:c r="U11"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>